<commit_message>
Completed version (still need to run again)
</commit_message>
<xml_diff>
--- a/Project/data/war_events.xlsx
+++ b/Project/data/war_events.xlsx
@@ -27,15 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>event_id</t>
   </si>
   <si>
     <t>event_name</t>
-  </si>
-  <si>
-    <t>event_name_cn</t>
   </si>
   <si>
     <t>start_date</t>
@@ -44,100 +41,25 @@
     <t>end_date</t>
   </si>
   <si>
-    <t>region</t>
+    <t>Iraq War</t>
   </si>
   <si>
-    <t>type</t>
+    <t>Lebanon War</t>
   </si>
   <si>
-    <t>intensity</t>
+    <t>Gaza War 2008</t>
   </si>
   <si>
-    <t>affected_assets</t>
+    <t>Gaza War 2014</t>
   </si>
   <si>
-    <t>Israel-Lebanon 2006</t>
+    <t>ISIS Iraq escalation</t>
   </si>
   <si>
-    <t>以色列-黎巴嫩战争</t>
+    <t>US-Iran crisis</t>
   </si>
   <si>
-    <t>Middle East</t>
-  </si>
-  <si>
-    <t>Interstate</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Gold,Oil,USD</t>
-  </si>
-  <si>
-    <t>Gaza Cast Lead 2008</t>
-  </si>
-  <si>
-    <t>以色列-加沙战争(铸铅行动)</t>
-  </si>
-  <si>
-    <t>Gold,Oil,EEM</t>
-  </si>
-  <si>
-    <t>Syria Civil War</t>
-  </si>
-  <si>
-    <t>叙利亚内战爆发</t>
-  </si>
-  <si>
-    <t>Civil War</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Oil,EEM</t>
-  </si>
-  <si>
-    <t>US-Iran Soleimani</t>
-  </si>
-  <si>
-    <t>美伊冲突/苏莱曼尼事件</t>
-  </si>
-  <si>
-    <t>Escalation</t>
-  </si>
-  <si>
-    <t>Gold,Oil,VIX</t>
-  </si>
-  <si>
-    <t>Israel-Hamas 2023</t>
-  </si>
-  <si>
-    <t>以色列-哈马斯战争</t>
-  </si>
-  <si>
-    <t>Israel-Iran Direct 2024</t>
-  </si>
-  <si>
-    <t>以色列-伊朗直接对抗</t>
-  </si>
-  <si>
-    <t>Extreme</t>
-  </si>
-  <si>
-    <t>Gold,Oil,DXY</t>
-  </si>
-  <si>
-    <t>Russia-Ukraine War</t>
-  </si>
-  <si>
-    <t>俄乌全面战争（对照组）</t>
-  </si>
-  <si>
-    <t>Europe</t>
-  </si>
-  <si>
-    <t>Gold,Oil,VIX,STOXX600</t>
+    <t>Israel-Hamas War</t>
   </si>
 </sst>
 </file>
@@ -753,12 +675,15 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1293,10 +1218,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I8"/>
-  <sheetFormatPr defaultColWidth="9.55752212389381" defaultRowHeight="13.5" outlineLevelRow="7"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="9.55752212389381" defaultRowHeight="13.5" outlineLevelRow="7" outlineLevelCol="3"/>
+  <cols>
+    <col min="2" max="2" width="22.4424778761062" customWidth="1"/>
+    <col min="3" max="3" width="11.7256637168142"/>
+    <col min="4" max="4" width="10.5929203539823"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1309,214 +1239,103 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
-      </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="1">
-        <v>38910</v>
-      </c>
-      <c r="E2" s="1">
-        <v>38943</v>
-      </c>
-      <c r="F2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I2" t="s">
-        <v>14</v>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>37700</v>
+      </c>
+      <c r="D2" s="2">
+        <v>37742</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="1">
-        <v>39809</v>
-      </c>
-      <c r="E3" s="1">
-        <v>39831</v>
-      </c>
-      <c r="F3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="2">
+        <v>38910</v>
+      </c>
+      <c r="D3" s="2">
+        <v>38943</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D4" s="1">
-        <v>40617</v>
-      </c>
-      <c r="F4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H4" t="s">
-        <v>21</v>
-      </c>
-      <c r="I4" t="s">
-        <v>22</v>
+      <c r="B4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2">
+        <v>39809</v>
+      </c>
+      <c r="D4" s="2">
+        <v>39831</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>23</v>
-      </c>
-      <c r="C5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="1">
-        <v>43833</v>
-      </c>
-      <c r="E5" s="1">
-        <v>43838</v>
-      </c>
-      <c r="F5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" t="s">
-        <v>26</v>
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="2">
+        <v>41828</v>
+      </c>
+      <c r="D5" s="2">
+        <v>41877</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" s="1">
-        <v>45206</v>
-      </c>
-      <c r="F6" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" t="s">
-        <v>17</v>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2">
+        <v>41800</v>
+      </c>
+      <c r="D6" s="2">
+        <v>41982</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:4">
       <c r="A7">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="1">
-        <v>45395</v>
-      </c>
-      <c r="E7" s="1">
-        <v>45591</v>
-      </c>
-      <c r="F7" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" t="s">
-        <v>31</v>
-      </c>
-      <c r="I7" t="s">
-        <v>32</v>
+      <c r="B7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="2">
+        <v>43833</v>
+      </c>
+      <c r="D7" s="2">
+        <v>43838</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:4">
       <c r="A8">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="1">
-        <v>44616</v>
-      </c>
-      <c r="F8" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" t="s">
-        <v>31</v>
-      </c>
-      <c r="I8" t="s">
-        <v>36</v>
+      <c r="B8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="2">
+        <v>45206</v>
+      </c>
+      <c r="D8" s="2">
+        <v>45310</v>
       </c>
     </row>
   </sheetData>

</xml_diff>